<commit_message>
Avancement du 14/08 et tests sur sortie Quarto (html simple ou via Quarto)
</commit_message>
<xml_diff>
--- a/02_data/Liste fichiers.xlsx
+++ b/02_data/Liste fichiers.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://agencesdeleau.sharepoint.com/sites/AESN-Etudespressions/Shared Documents/Pressions/PANDA Pression/02_data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://agencesdeleau.sharepoint.com/sites/AESN-Etudespressions/Shared Documents/Pressions/PANDA Pression/PANDA_Pression/02_data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="16" documentId="8_{9F15B30D-45CF-4112-AFE5-971E02649CE4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{007D6E97-E801-41DE-93F4-E5715AE92554}"/>
+  <xr:revisionPtr revIDLastSave="17" documentId="8_{9F15B30D-45CF-4112-AFE5-971E02649CE4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{26AC7261-A766-4A2E-9673-9076B87450CB}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{64C32074-7079-410A-A620-303E49B92065}"/>
   </bookViews>
@@ -65,9 +65,6 @@
     <t>EDL</t>
   </si>
   <si>
-    <t>Table_Param_Unités.xlsx</t>
-  </si>
-  <si>
     <t>Table desparamètres et unités standards utilisés dans PANDA Pression.</t>
   </si>
   <si>
@@ -114,6 +111,9 @@
   </si>
   <si>
     <t>Table des débits de référence par tronçon de masse d'eau à utiliser pour l'étude</t>
+  </si>
+  <si>
+    <t>Table_Param_Unites.xlsx</t>
   </si>
 </sst>
 </file>
@@ -516,10 +516,10 @@
         <v>4</v>
       </c>
       <c r="B2" t="s">
+        <v>24</v>
+      </c>
+      <c r="C2" t="s">
         <v>8</v>
-      </c>
-      <c r="C2" t="s">
-        <v>9</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
@@ -528,7 +528,7 @@
       </c>
       <c r="B3" s="1"/>
       <c r="C3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
@@ -536,10 +536,10 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C4" t="s">
         <v>10</v>
-      </c>
-      <c r="C4" t="s">
-        <v>11</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.3">
@@ -547,10 +547,10 @@
         <v>6</v>
       </c>
       <c r="B6" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C6" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.3">
@@ -558,10 +558,10 @@
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C7" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.3">
@@ -569,10 +569,10 @@
         <v>7</v>
       </c>
       <c r="B8" t="s">
+        <v>15</v>
+      </c>
+      <c r="C8" t="s">
         <v>16</v>
-      </c>
-      <c r="C8" t="s">
-        <v>17</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.3">
@@ -580,10 +580,10 @@
         <v>7</v>
       </c>
       <c r="B9" t="s">
+        <v>17</v>
+      </c>
+      <c r="C9" t="s">
         <v>18</v>
-      </c>
-      <c r="C9" t="s">
-        <v>19</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.3">
@@ -591,7 +591,7 @@
         <v>5</v>
       </c>
       <c r="B12" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.3">
@@ -599,7 +599,7 @@
         <v>5</v>
       </c>
       <c r="B13" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.3">
@@ -607,7 +607,7 @@
         <v>5</v>
       </c>
       <c r="B14" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.3">
@@ -616,7 +616,7 @@
       </c>
       <c r="B15" s="1"/>
       <c r="C15" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
   </sheetData>
@@ -625,6 +625,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100E0B707973A0EDF4D8C0132D38830BF56" ma:contentTypeVersion="3" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="6fab73de96728382b95836a8b817e49f">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="4222387a-a7c4-4a56-bf01-5dca1ac56634" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="2d5a3db95c4c940e29da1a6f70bc1044" ns2:_="">
     <xsd:import namespace="4222387a-a7c4-4a56-bf01-5dca1ac56634"/>
@@ -762,15 +771,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement/>
@@ -778,13 +778,22 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3DF59F40-9F75-41DC-A729-F5EE6AF66A55}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C6773EF1-3CA8-427C-B3DF-0D622DE2A109}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C6773EF1-3CA8-427C-B3DF-0D622DE2A109}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{776A37C3-553D-4BD3-B115-DF7D653C6AF9}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{609A8DBE-E0F8-450C-90B7-A722ECCA9954}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{609A8DBE-E0F8-450C-90B7-A722ECCA9954}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>